<commit_message>
fix: restore light mode toggle, dark default theme, navbar theme-aware, XLSX template
- Fix light mode CSS: replace html.light (never set by next-themes) with html:not(.dark)
- Set defaultTheme=dark in ThemeProvider since spec mandates dark background
- Navbar uses semantic theme CSS variables (border-border, bg-card, text-foreground, text-muted-foreground)
- Add Zynqio_Template.xlsx to public/ for static download link in import modal
- Build: 33 pages, 0 errors

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Zynqio_Template.xlsx
+++ b/public/Zynqio_Template.xlsx
@@ -397,32 +397,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Question</v>
+        <v>question</v>
       </c>
       <c r="B1" t="str">
-        <v>Type</v>
+        <v>type</v>
       </c>
       <c r="C1" t="str">
-        <v>Option A</v>
+        <v>option_a</v>
       </c>
       <c r="D1" t="str">
-        <v>Option B</v>
+        <v>option_b</v>
       </c>
       <c r="E1" t="str">
-        <v>Option C</v>
+        <v>option_c</v>
       </c>
       <c r="F1" t="str">
-        <v>Option D</v>
+        <v>option_d</v>
       </c>
       <c r="G1" t="str">
-        <v>Correct Answer</v>
+        <v>correct_answer</v>
       </c>
       <c r="H1" t="str">
-        <v>Points</v>
+        <v>points</v>
+      </c>
+      <c r="I1" t="str">
+        <v>time_override</v>
       </c>
     </row>
     <row r="2">
@@ -450,10 +453,13 @@
       <c r="H2" t="str">
         <v>1</v>
       </c>
+      <c r="I2" t="str">
+        <v>30</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Is the Earth flat?</v>
+        <v>Bumi lebih besar dari Bulan.</v>
       </c>
       <c r="B3" t="str">
         <v>TF</v>
@@ -471,10 +477,13 @@
         <v/>
       </c>
       <c r="G3" t="str">
-        <v>B</v>
+        <v>TRUE</v>
       </c>
       <c r="H3" t="str">
         <v>1</v>
+      </c>
+      <c r="I3" t="str">
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -502,6 +511,9 @@
       <c r="H4" t="str">
         <v>1</v>
       </c>
+      <c r="I4" t="str">
+        <v>15</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -528,10 +540,42 @@
       <c r="H5" t="str">
         <v>1</v>
       </c>
+      <c r="I5" t="str">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Explain the water cycle in your own words.</v>
+      </c>
+      <c r="B6" t="str">
+        <v>OPEN</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>2</v>
+      </c>
+      <c r="I6" t="str">
+        <v>120</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>